<commit_message>
Include received 1Q26 inputs and preserve 4Q25 regression fixtures
</commit_message>
<xml_diff>
--- a/inputs/allocation_history.xlsx
+++ b/inputs/allocation_history.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -475,7 +475,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>480</v>
+        <v>496</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>372</v>
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>482</v>
+        <v>498</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>386</v>
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>484</v>
+        <v>500</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>397</v>
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>486</v>
+        <v>502</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>405</v>
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>489</v>
+        <v>505</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>412</v>
@@ -540,10 +540,10 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>491</v>
+        <v>508</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>424</v>
+        <v>419</v>
       </c>
     </row>
     <row r="8">
@@ -553,10 +553,10 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>489</v>
+        <v>510</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>437</v>
+        <v>428</v>
       </c>
     </row>
     <row r="9">
@@ -566,10 +566,23 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>496</v>
+        <v>512</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>436</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1Q26</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>515</v>
+      </c>
+      <c r="C10" t="n">
+        <v>457</v>
       </c>
     </row>
   </sheetData>

</xml_diff>